<commit_message>
Describe changes (e.g. add port fallback in app.py)
</commit_message>
<xml_diff>
--- a/emails.xlsx
+++ b/emails.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Emails" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3043,8 +3043,16 @@
           <t>Evea Urora</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>16401657</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>MBUGUA GITAU LTD</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">

</xml_diff>